<commit_message>
3.1.33 Adapt MethodMetaInfo for service method.
</commit_message>
<xml_diff>
--- a/meta/program/BlancoRestGeneratorKtResourceBundle.xlsx
+++ b/meta/program/BlancoRestGeneratorKtResourceBundle.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tueda/data/webstorm/blanco/blancoRestGeneratorKt/meta/program/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45C446B2-1161-0C42-934F-5B9149D53E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B1E38D-A846-7745-9F47-1DFE8C23D7FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="840" yWindow="500" windowWidth="27640" windowHeight="19980" tabRatio="640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="203">
   <si>
     <t>リソースバンドル定義書</t>
   </si>
@@ -1219,6 +1219,14 @@
   </si>
   <si>
     <t>META2XML.PROCESS_COMMOINTERFACE</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>META2XML.PROCESS_METHODINFO</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>blancotelegramprocess-methodinfo</t>
     <phoneticPr fontId="4"/>
   </si>
 </sst>
@@ -2084,7 +2092,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I128"/>
+  <dimension ref="A1:I129"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
@@ -2692,10 +2700,10 @@
         <v>28</v>
       </c>
       <c r="B42" s="22" t="s">
-        <v>136</v>
+        <v>201</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>140</v>
+        <v>202</v>
       </c>
       <c r="D42" s="24"/>
       <c r="E42" s="24"/>
@@ -2710,10 +2718,10 @@
         <v>29</v>
       </c>
       <c r="B43" s="22" t="s">
-        <v>63</v>
+        <v>136</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>62</v>
+        <v>140</v>
       </c>
       <c r="D43" s="24"/>
       <c r="E43" s="24"/>
@@ -2722,22 +2730,23 @@
       <c r="H43" s="25"/>
       <c r="I43" s="16"/>
     </row>
-    <row r="44" spans="1:9" s="34" customFormat="1">
+    <row r="44" spans="1:9">
       <c r="A44" s="21">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="B44" s="33" t="s">
-        <v>109</v>
-      </c>
-      <c r="C44" s="38" t="s">
-        <v>110</v>
-      </c>
-      <c r="D44" s="39"/>
-      <c r="E44" s="39"/>
-      <c r="F44" s="39"/>
-      <c r="G44" s="39"/>
+      <c r="B44" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C44" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="D44" s="24"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="24"/>
+      <c r="G44" s="24"/>
       <c r="H44" s="25"/>
+      <c r="I44" s="16"/>
     </row>
     <row r="45" spans="1:9" s="34" customFormat="1">
       <c r="A45" s="21">
@@ -2745,10 +2754,10 @@
         <v>31</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C45" s="38" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D45" s="39"/>
       <c r="E45" s="39"/>
@@ -2762,10 +2771,10 @@
         <v>32</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C46" s="38" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D46" s="39"/>
       <c r="E46" s="39"/>
@@ -2779,10 +2788,10 @@
         <v>33</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C47" s="38" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D47" s="39"/>
       <c r="E47" s="39"/>
@@ -2796,10 +2805,10 @@
         <v>34</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C48" s="38" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D48" s="39"/>
       <c r="E48" s="39"/>
@@ -2813,10 +2822,10 @@
         <v>35</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C49" s="38" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D49" s="39"/>
       <c r="E49" s="39"/>
@@ -2830,10 +2839,10 @@
         <v>36</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C50" s="38" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D50" s="39"/>
       <c r="E50" s="39"/>
@@ -2847,30 +2856,33 @@
         <v>37</v>
       </c>
       <c r="B51" s="33" t="s">
+        <v>121</v>
+      </c>
+      <c r="C51" s="38" t="s">
+        <v>122</v>
+      </c>
+      <c r="D51" s="39"/>
+      <c r="E51" s="39"/>
+      <c r="F51" s="39"/>
+      <c r="G51" s="39"/>
+      <c r="H51" s="25"/>
+    </row>
+    <row r="52" spans="1:9" s="34" customFormat="1">
+      <c r="A52" s="21">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="B52" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="C51" s="35" t="s">
+      <c r="C52" s="35" t="s">
         <v>124</v>
       </c>
-      <c r="D51" s="36"/>
-      <c r="E51" s="36"/>
-      <c r="F51" s="36"/>
-      <c r="G51" s="37"/>
-      <c r="H51" s="25"/>
-    </row>
-    <row r="52" spans="1:9">
-      <c r="A52" s="21">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-      <c r="B52" s="22"/>
-      <c r="C52" s="23"/>
-      <c r="D52" s="24"/>
-      <c r="E52" s="24"/>
-      <c r="F52" s="24"/>
-      <c r="G52" s="24"/>
+      <c r="D52" s="36"/>
+      <c r="E52" s="36"/>
+      <c r="F52" s="36"/>
+      <c r="G52" s="37"/>
       <c r="H52" s="25"/>
-      <c r="I52" s="16"/>
     </row>
     <row r="53" spans="1:9">
       <c r="A53" s="21">
@@ -2878,9 +2890,7 @@
         <v>39</v>
       </c>
       <c r="B53" s="22"/>
-      <c r="C53" s="23" t="s">
-        <v>18</v>
-      </c>
+      <c r="C53" s="23"/>
       <c r="D53" s="24"/>
       <c r="E53" s="24"/>
       <c r="F53" s="24"/>
@@ -2893,11 +2903,9 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="B54" s="22" t="s">
-        <v>22</v>
-      </c>
+      <c r="B54" s="22"/>
       <c r="C54" s="23" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D54" s="24"/>
       <c r="E54" s="24"/>
@@ -2912,10 +2920,10 @@
         <v>41</v>
       </c>
       <c r="B55" s="22" t="s">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="C55" s="23" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="D55" s="24"/>
       <c r="E55" s="24"/>
@@ -2930,10 +2938,10 @@
         <v>42</v>
       </c>
       <c r="B56" s="22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C56" s="23" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="D56" s="24"/>
       <c r="E56" s="24"/>
@@ -2948,10 +2956,10 @@
         <v>43</v>
       </c>
       <c r="B57" s="22" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D57" s="24"/>
       <c r="E57" s="24"/>
@@ -2966,10 +2974,10 @@
         <v>44</v>
       </c>
       <c r="B58" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C58" s="23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D58" s="24"/>
       <c r="E58" s="24"/>
@@ -2984,10 +2992,10 @@
         <v>45</v>
       </c>
       <c r="B59" s="22" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="C59" s="23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D59" s="24"/>
       <c r="E59" s="24"/>
@@ -3002,10 +3010,10 @@
         <v>46</v>
       </c>
       <c r="B60" s="22" t="s">
-        <v>141</v>
+        <v>55</v>
       </c>
       <c r="C60" s="23" t="s">
-        <v>143</v>
+        <v>32</v>
       </c>
       <c r="D60" s="24"/>
       <c r="E60" s="24"/>
@@ -3020,10 +3028,10 @@
         <v>47</v>
       </c>
       <c r="B61" s="22" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C61" s="23" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D61" s="24"/>
       <c r="E61" s="24"/>
@@ -3038,10 +3046,10 @@
         <v>48</v>
       </c>
       <c r="B62" s="22" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C62" s="23" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D62" s="24"/>
       <c r="E62" s="24"/>
@@ -3055,8 +3063,12 @@
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-      <c r="B63" s="22"/>
-      <c r="C63" s="23"/>
+      <c r="B63" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="C63" s="23" t="s">
+        <v>145</v>
+      </c>
       <c r="D63" s="24"/>
       <c r="E63" s="24"/>
       <c r="F63" s="24"/>
@@ -3069,12 +3081,8 @@
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="B64" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="C64" s="23" t="s">
-        <v>41</v>
-      </c>
+      <c r="B64" s="22"/>
+      <c r="C64" s="23"/>
       <c r="D64" s="24"/>
       <c r="E64" s="24"/>
       <c r="F64" s="24"/>
@@ -3088,10 +3096,10 @@
         <v>51</v>
       </c>
       <c r="B65" s="22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C65" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D65" s="24"/>
       <c r="E65" s="24"/>
@@ -3106,10 +3114,10 @@
         <v>52</v>
       </c>
       <c r="B66" s="22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C66" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D66" s="24"/>
       <c r="E66" s="24"/>
@@ -3123,8 +3131,12 @@
         <f t="shared" si="0"/>
         <v>53</v>
       </c>
-      <c r="B67" s="22"/>
-      <c r="C67" s="23"/>
+      <c r="B67" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C67" s="23" t="s">
+        <v>43</v>
+      </c>
       <c r="D67" s="24"/>
       <c r="E67" s="24"/>
       <c r="F67" s="24"/>
@@ -3137,12 +3149,8 @@
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="B68" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C68" s="23" t="s">
-        <v>44</v>
-      </c>
+      <c r="B68" s="22"/>
+      <c r="C68" s="23"/>
       <c r="D68" s="24"/>
       <c r="E68" s="24"/>
       <c r="F68" s="24"/>
@@ -3156,10 +3164,10 @@
         <v>55</v>
       </c>
       <c r="B69" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="C69" s="26" t="s">
-        <v>42</v>
+        <v>38</v>
+      </c>
+      <c r="C69" s="23" t="s">
+        <v>44</v>
       </c>
       <c r="D69" s="24"/>
       <c r="E69" s="24"/>
@@ -3174,10 +3182,10 @@
         <v>56</v>
       </c>
       <c r="B70" s="22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C70" s="26" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D70" s="24"/>
       <c r="E70" s="24"/>
@@ -3191,8 +3199,12 @@
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
-      <c r="B71" s="22"/>
-      <c r="C71" s="26"/>
+      <c r="B71" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="C71" s="26" t="s">
+        <v>45</v>
+      </c>
       <c r="D71" s="24"/>
       <c r="E71" s="24"/>
       <c r="F71" s="24"/>
@@ -3205,12 +3217,8 @@
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="B72" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="C72" s="26" t="s">
-        <v>50</v>
-      </c>
+      <c r="B72" s="22"/>
+      <c r="C72" s="26"/>
       <c r="D72" s="24"/>
       <c r="E72" s="24"/>
       <c r="F72" s="24"/>
@@ -3224,10 +3232,10 @@
         <v>59</v>
       </c>
       <c r="B73" s="22" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C73" s="26" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="D73" s="24"/>
       <c r="E73" s="24"/>
@@ -3242,10 +3250,10 @@
         <v>60</v>
       </c>
       <c r="B74" s="22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C74" s="26" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D74" s="24"/>
       <c r="E74" s="24"/>
@@ -3260,10 +3268,10 @@
         <v>61</v>
       </c>
       <c r="B75" s="22" t="s">
-        <v>49</v>
-      </c>
-      <c r="C75" s="32" t="s">
-        <v>51</v>
+        <v>48</v>
+      </c>
+      <c r="C75" s="26" t="s">
+        <v>43</v>
       </c>
       <c r="D75" s="24"/>
       <c r="E75" s="24"/>
@@ -3277,8 +3285,12 @@
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
-      <c r="B76" s="22"/>
-      <c r="C76" s="26"/>
+      <c r="B76" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="C76" s="32" t="s">
+        <v>51</v>
+      </c>
       <c r="D76" s="24"/>
       <c r="E76" s="24"/>
       <c r="F76" s="24"/>
@@ -3291,12 +3303,8 @@
         <f t="shared" si="0"/>
         <v>63</v>
       </c>
-      <c r="B77" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="C77" s="23" t="s">
-        <v>86</v>
-      </c>
+      <c r="B77" s="22"/>
+      <c r="C77" s="26"/>
       <c r="D77" s="24"/>
       <c r="E77" s="24"/>
       <c r="F77" s="24"/>
@@ -3310,10 +3318,10 @@
         <v>64</v>
       </c>
       <c r="B78" s="22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C78" s="23" t="s">
-        <v>42</v>
+        <v>86</v>
       </c>
       <c r="D78" s="24"/>
       <c r="E78" s="24"/>
@@ -3328,10 +3336,10 @@
         <v>65</v>
       </c>
       <c r="B79" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="C79" s="26" t="s">
-        <v>43</v>
+        <v>83</v>
+      </c>
+      <c r="C79" s="23" t="s">
+        <v>42</v>
       </c>
       <c r="D79" s="24"/>
       <c r="E79" s="24"/>
@@ -3346,10 +3354,10 @@
         <v>66</v>
       </c>
       <c r="B80" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="C80" s="31" t="s">
-        <v>87</v>
+        <v>84</v>
+      </c>
+      <c r="C80" s="26" t="s">
+        <v>43</v>
       </c>
       <c r="D80" s="24"/>
       <c r="E80" s="24"/>
@@ -3360,11 +3368,15 @@
     </row>
     <row r="81" spans="1:9">
       <c r="A81" s="21">
-        <f t="shared" ref="A81:A128" si="1">A80+1</f>
+        <f t="shared" ref="A81:A129" si="1">A80+1</f>
         <v>67</v>
       </c>
-      <c r="B81" s="22"/>
-      <c r="C81" s="26"/>
+      <c r="B81" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C81" s="31" t="s">
+        <v>87</v>
+      </c>
       <c r="D81" s="24"/>
       <c r="E81" s="24"/>
       <c r="F81" s="24"/>
@@ -3377,12 +3389,8 @@
         <f t="shared" si="1"/>
         <v>68</v>
       </c>
-      <c r="B82" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="C82" s="23" t="s">
-        <v>17</v>
-      </c>
+      <c r="B82" s="22"/>
+      <c r="C82" s="26"/>
       <c r="D82" s="24"/>
       <c r="E82" s="24"/>
       <c r="F82" s="24"/>
@@ -3396,10 +3404,10 @@
         <v>69</v>
       </c>
       <c r="B83" s="22" t="s">
-        <v>152</v>
+        <v>21</v>
       </c>
       <c r="C83" s="23" t="s">
-        <v>153</v>
+        <v>17</v>
       </c>
       <c r="D83" s="24"/>
       <c r="E83" s="24"/>
@@ -3413,25 +3421,31 @@
         <f t="shared" si="1"/>
         <v>70</v>
       </c>
-      <c r="B84" s="27"/>
-      <c r="C84" s="28"/>
-      <c r="D84" s="29"/>
-      <c r="E84" s="29"/>
-      <c r="F84" s="29"/>
-      <c r="G84" s="29"/>
-      <c r="H84" s="30"/>
+      <c r="B84" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="C84" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="D84" s="24"/>
+      <c r="E84" s="24"/>
+      <c r="F84" s="24"/>
+      <c r="G84" s="24"/>
+      <c r="H84" s="25"/>
+      <c r="I84" s="16"/>
     </row>
     <row r="85" spans="1:9">
       <c r="A85" s="21">
         <f t="shared" si="1"/>
         <v>71</v>
       </c>
-      <c r="B85" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>65</v>
-      </c>
+      <c r="B85" s="27"/>
+      <c r="C85" s="28"/>
+      <c r="D85" s="29"/>
+      <c r="E85" s="29"/>
+      <c r="F85" s="29"/>
+      <c r="G85" s="29"/>
+      <c r="H85" s="30"/>
     </row>
     <row r="86" spans="1:9">
       <c r="A86" s="21">
@@ -3439,10 +3453,10 @@
         <v>72</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="87" spans="1:9">
@@ -3451,10 +3465,10 @@
         <v>73</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>190</v>
+        <v>66</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>187</v>
+        <v>69</v>
       </c>
     </row>
     <row r="88" spans="1:9">
@@ -3463,10 +3477,10 @@
         <v>74</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="89" spans="1:9">
@@ -3475,10 +3489,10 @@
         <v>75</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="90" spans="1:9">
@@ -3487,10 +3501,10 @@
         <v>76</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>67</v>
+        <v>192</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>68</v>
+        <v>189</v>
       </c>
     </row>
     <row r="91" spans="1:9">
@@ -3499,10 +3513,10 @@
         <v>77</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="92" spans="1:9">
@@ -3511,10 +3525,10 @@
         <v>78</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="93" spans="1:9">
@@ -3523,10 +3537,10 @@
         <v>79</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="94" spans="1:9">
@@ -3535,10 +3549,10 @@
         <v>80</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="95" spans="1:9">
@@ -3547,10 +3561,10 @@
         <v>81</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>193</v>
+        <v>75</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>194</v>
+        <v>77</v>
       </c>
     </row>
     <row r="96" spans="1:9">
@@ -3559,10 +3573,10 @@
         <v>82</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -3571,10 +3585,10 @@
         <v>83</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -3583,10 +3597,10 @@
         <v>84</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>156</v>
+        <v>197</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>157</v>
+        <v>198</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -3595,10 +3609,10 @@
         <v>85</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -3607,10 +3621,10 @@
         <v>86</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -3619,10 +3633,10 @@
         <v>87</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>79</v>
+        <v>158</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>78</v>
+        <v>159</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -3631,7 +3645,7 @@
         <v>88</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>78</v>
@@ -3643,10 +3657,10 @@
         <v>89</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -3655,7 +3669,7 @@
         <v>90</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>92</v>
@@ -3667,10 +3681,10 @@
         <v>91</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -3679,7 +3693,7 @@
         <v>92</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>93</v>
@@ -3690,18 +3704,18 @@
         <f t="shared" si="1"/>
         <v>93</v>
       </c>
+      <c r="B107" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" s="21">
         <f t="shared" si="1"/>
         <v>94</v>
       </c>
-      <c r="B108" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="C108" s="1" t="s">
-        <v>181</v>
-      </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" s="21">
@@ -3709,10 +3723,10 @@
         <v>95</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -3721,10 +3735,10 @@
         <v>96</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="111" spans="1:3">
@@ -3733,10 +3747,10 @@
         <v>97</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>96</v>
+        <v>183</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -3745,10 +3759,10 @@
         <v>98</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -3757,10 +3771,10 @@
         <v>99</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>150</v>
+        <v>99</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>184</v>
+        <v>100</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -3769,10 +3783,10 @@
         <v>100</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -3781,10 +3795,10 @@
         <v>101</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -3793,10 +3807,10 @@
         <v>102</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -3805,10 +3819,10 @@
         <v>103</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -3817,10 +3831,10 @@
         <v>104</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -3828,18 +3842,18 @@
         <f t="shared" si="1"/>
         <v>105</v>
       </c>
+      <c r="B119" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" s="21">
         <f t="shared" si="1"/>
         <v>106</v>
       </c>
-      <c r="B120" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C120" s="1" t="s">
-        <v>125</v>
-      </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" s="21">
@@ -3847,10 +3861,10 @@
         <v>107</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="122" spans="1:3">
@@ -3858,18 +3872,18 @@
         <f t="shared" si="1"/>
         <v>108</v>
       </c>
+      <c r="B122" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" s="21">
         <f t="shared" si="1"/>
         <v>109</v>
       </c>
-      <c r="B123" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="C123" s="1" t="s">
-        <v>161</v>
-      </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" s="21">
@@ -3877,10 +3891,10 @@
         <v>110</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="125" spans="1:3">
@@ -3889,10 +3903,10 @@
         <v>111</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="126" spans="1:3">
@@ -3901,10 +3915,10 @@
         <v>112</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
     </row>
     <row r="127" spans="1:3">
@@ -3913,10 +3927,10 @@
         <v>113</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="128" spans="1:3">
@@ -3925,9 +3939,21 @@
         <v>114</v>
       </c>
       <c r="B128" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3">
+      <c r="A129" s="21">
+        <f t="shared" si="1"/>
+        <v>115</v>
+      </c>
+      <c r="B129" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C128" s="1" t="s">
+      <c r="C129" s="1" t="s">
         <v>179</v>
       </c>
     </row>
@@ -3939,7 +3965,7 @@
   </mergeCells>
   <phoneticPr fontId="4"/>
   <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D120:D121 D111:D118" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D121:D122 D112:D119" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>型</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>